<commit_message>
Improve background (UI) and add CSV as a source of vendors. Do not touch vendors list, as it's a source of truth file.
</commit_message>
<xml_diff>
--- a/server/data/Vendor List.xlsx
+++ b/server/data/Vendor List.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A9"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -439,9 +439,14 @@
         <v>Services, Inc.</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Account#: 5653</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A9"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>